<commit_message>
update indices de precios
</commit_message>
<xml_diff>
--- a/data/analysis-data/20260605_panel_eaae.xlsx
+++ b/data/analysis-data/20260605_panel_eaae.xlsx
@@ -1618,7 +1618,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Oyanthabal; usado para costo_laboral.</t>
+          <t>Oyanthabal; usado para costo_laboral. Si la planilla no lo trae explícito, se deriva desde ipc_index_1983_1989 normalizando 2005=1.</t>
         </is>
       </c>
     </row>
@@ -3638,99 +3638,65 @@
       <c r="D21">
         <v>6.6</v>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E21">
+        <v>3.07205708091106</v>
       </c>
       <c r="F21">
         <v>3.14718882182406</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G21">
+        <v>195574988539.379</v>
+      </c>
+      <c r="H21">
+        <v>59557197640.5947</v>
+      </c>
+      <c r="I21">
+        <v>272887536854.195</v>
+      </c>
+      <c r="J21">
+        <v>49283163317.2784</v>
+      </c>
+      <c r="K21">
+        <v>6428762644.43935</v>
       </c>
       <c r="L21">
         <v>24872424541.7009</v>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M21">
+        <v>96457387673.0094</v>
+      </c>
+      <c r="N21">
+        <v>96457387673.0094</v>
       </c>
       <c r="O21">
         <v>84764.4647407208</v>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="P21">
+        <v>17981976131.1382</v>
+      </c>
+      <c r="Q21">
+        <v>28256010454.4544</v>
+      </c>
+      <c r="R21">
+        <v>136017790898.784</v>
+      </c>
+      <c r="S21">
+        <v>24377305369.7704</v>
+      </c>
+      <c r="T21">
+        <v>120834693042.78</v>
+      </c>
+      <c r="U21">
+        <v>0.14881467961169</v>
+      </c>
+      <c r="V21">
+        <v>0.233840213790677</v>
+      </c>
+      <c r="W21">
+        <v>0.218248141073648</v>
+      </c>
+      <c r="X21">
+        <v>702619.875236272</v>
       </c>
     </row>
     <row r="22">
@@ -3750,99 +3716,65 @@
       <c r="D22">
         <v>6.6</v>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E22">
+        <v>3.41225692935307</v>
       </c>
       <c r="F22">
         <v>3.39769972910033</v>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G22">
+        <v>216997552005.529</v>
+      </c>
+      <c r="H22">
+        <v>65931342445.5778</v>
+      </c>
+      <c r="I22">
+        <v>297794919014.519</v>
+      </c>
+      <c r="J22">
+        <v>62727489228.5619</v>
+      </c>
+      <c r="K22">
+        <v>6370954532.13645</v>
       </c>
       <c r="L22">
         <v>24758544187.2287</v>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M22">
+        <v>110540909913.194</v>
+      </c>
+      <c r="N22">
+        <v>110540909913.194</v>
       </c>
       <c r="O22">
         <v>86333.0943782653</v>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="P22">
+        <v>31597990509.1967</v>
+      </c>
+      <c r="Q22">
+        <v>34801843726.2126</v>
+      </c>
+      <c r="R22">
+        <v>151066209559.952</v>
+      </c>
+      <c r="S22">
+        <v>26640114204.1182</v>
+      </c>
+      <c r="T22">
+        <v>137181024117.312</v>
+      </c>
+      <c r="U22">
+        <v>0.230337910891927</v>
+      </c>
+      <c r="V22">
+        <v>0.253692840902335</v>
+      </c>
+      <c r="W22">
+        <v>0.221398480080727</v>
+      </c>
+      <c r="X22">
+        <v>763685.616974436</v>
       </c>
     </row>
     <row r="23">
@@ -3862,99 +3794,65 @@
       <c r="D23">
         <v>6.6</v>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E23">
+        <v>3.61661765851799</v>
       </c>
       <c r="F23">
         <v>3.70010931039399</v>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G23">
+        <v>245380682520.025</v>
+      </c>
+      <c r="H23">
+        <v>73421100951.1512</v>
+      </c>
+      <c r="I23">
+        <v>299334834599.419</v>
+      </c>
+      <c r="J23">
+        <v>62298329349.3866</v>
+      </c>
+      <c r="K23">
+        <v>5951262672.89858</v>
       </c>
       <c r="L23">
         <v>25839753913.5667</v>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M23">
+        <v>108555428018.29</v>
+      </c>
+      <c r="N23">
+        <v>108555428018.29</v>
       </c>
       <c r="O23">
         <v>89467.5060887856</v>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="P23">
+        <v>30507312762.9213</v>
+      </c>
+      <c r="Q23">
+        <v>41630084364.6859</v>
+      </c>
+      <c r="R23">
+        <v>171959581568.874</v>
+      </c>
+      <c r="S23">
+        <v>29969596285.2183</v>
+      </c>
+      <c r="T23">
+        <v>138525024303.508</v>
+      </c>
+      <c r="U23">
+        <v>0.220229614947259</v>
+      </c>
+      <c r="V23">
+        <v>0.300523927528606</v>
+      </c>
+      <c r="W23">
+        <v>0.245280844273958</v>
+      </c>
+      <c r="X23">
+        <v>820645.440572465</v>
       </c>
     </row>
     <row r="24">
@@ -3974,99 +3872,65 @@
       <c r="D24">
         <v>6.6</v>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E24">
+        <v>3.76320113204531</v>
       </c>
       <c r="F24">
         <v>3.88878855567701</v>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G24">
+        <v>215133997424.447</v>
+      </c>
+      <c r="H24">
+        <v>63809281335.2196</v>
+      </c>
+      <c r="I24">
+        <v>303932409821.641</v>
+      </c>
+      <c r="J24">
+        <v>52731349214.1726</v>
+      </c>
+      <c r="K24">
+        <v>6559395292.76757</v>
       </c>
       <c r="L24">
         <v>26902928344.787</v>
       </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M24">
+        <v>106946925737.8</v>
+      </c>
+      <c r="N24">
+        <v>106946925737.8</v>
       </c>
       <c r="O24">
         <v>89501.9413936812</v>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="P24">
+        <v>19269025576.618</v>
+      </c>
+      <c r="Q24">
+        <v>30346957697.665</v>
+      </c>
+      <c r="R24">
+        <v>151324716089.228</v>
+      </c>
+      <c r="S24">
+        <v>27004188550.6083</v>
+      </c>
+      <c r="T24">
+        <v>133951114288.408</v>
+      </c>
+      <c r="U24">
+        <v>0.143851177938917</v>
+      </c>
+      <c r="V24">
+        <v>0.226552484157209</v>
+      </c>
+      <c r="W24">
+        <v>0.209945630255968</v>
+      </c>
+      <c r="X24">
+        <v>712937.39936377</v>
       </c>
     </row>
     <row r="25">
@@ -4086,99 +3950,65 @@
       <c r="D25">
         <v>6.6</v>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E25">
+        <v>3.92076753234211</v>
       </c>
       <c r="F25">
         <v>4.1023240340288</v>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G25">
+        <v>218852967067.022</v>
+      </c>
+      <c r="H25">
+        <v>67326186301.5835</v>
+      </c>
+      <c r="I25">
+        <v>320611447753.721</v>
+      </c>
+      <c r="J25">
+        <v>55754572590.0453</v>
+      </c>
+      <c r="K25">
+        <v>7017952212.74117</v>
       </c>
       <c r="L25">
         <v>27526900531.3037</v>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M25">
+        <v>111449085921.908</v>
+      </c>
+      <c r="N25">
+        <v>111449085921.908</v>
       </c>
       <c r="O25">
         <v>90863.9271580213</v>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="P25">
+        <v>21209719846.0005</v>
+      </c>
+      <c r="Q25">
+        <v>32781333557.5386</v>
+      </c>
+      <c r="R25">
+        <v>151526780765.439</v>
+      </c>
+      <c r="S25">
+        <v>27129345651.0216</v>
+      </c>
+      <c r="T25">
+        <v>138578431572.93</v>
+      </c>
+      <c r="U25">
+        <v>0.153052099127262</v>
+      </c>
+      <c r="V25">
+        <v>0.236554369864453</v>
+      </c>
+      <c r="W25">
+        <v>0.209993082821236</v>
+      </c>
+      <c r="X25">
+        <v>740956.157271263</v>
       </c>
     </row>
   </sheetData>
@@ -5536,81 +5366,53 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D21">
+        <v>-8.9488630561202</v>
+      </c>
+      <c r="E21">
+        <v>-8.14977168410478</v>
+      </c>
+      <c r="F21">
+        <v>-8.61129634475476</v>
+      </c>
+      <c r="G21">
+        <v>-4.76250800825247</v>
       </c>
       <c r="H21">
         <v>-10.70273347017</v>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="I21">
+        <v>-5.42650032789647</v>
+      </c>
+      <c r="J21">
+        <v>-5.42650032789647</v>
       </c>
       <c r="K21">
         <v>-6.81276745254741</v>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L21">
+        <v>-6.15774093010633</v>
+      </c>
+      <c r="M21">
+        <v>-5.32655285542266</v>
+      </c>
+      <c r="N21">
+        <v>-9.63061786909387</v>
+      </c>
+      <c r="O21">
+        <v>-9.96613121609577</v>
+      </c>
+      <c r="P21">
+        <v>-6.56864371252708</v>
+      </c>
+      <c r="Q21">
+        <v>0.439791092357122</v>
+      </c>
+      <c r="R21">
+        <v>1.32941541946872</v>
+      </c>
+      <c r="S21">
+        <v>-1.43475044274605</v>
       </c>
     </row>
     <row r="22">
@@ -5627,81 +5429,53 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D22">
+        <v>8.41214036892506</v>
+      </c>
+      <c r="E22">
+        <v>9.1273432445663</v>
+      </c>
+      <c r="F22">
+        <v>14.5082461314175</v>
+      </c>
+      <c r="G22">
+        <v>-8.31829748117038</v>
       </c>
       <c r="H22">
         <v>-2.29633586452175</v>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="I22">
+        <v>1.28923469597375</v>
+      </c>
+      <c r="J22">
+        <v>1.28923469597375</v>
       </c>
       <c r="K22">
         <v>5.73922499549879</v>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L22">
+        <v>46.7881011589845</v>
+      </c>
+      <c r="M22">
+        <v>27.979736622065</v>
+      </c>
+      <c r="N22">
+        <v>7.79195723640211</v>
+      </c>
+      <c r="O22">
+        <v>4.66070444869062</v>
+      </c>
+      <c r="P22">
+        <v>2.10663089349425</v>
+      </c>
+      <c r="Q22">
+        <v>43.7596166620136</v>
+      </c>
+      <c r="R22">
+        <v>25.3393002023136</v>
+      </c>
+      <c r="S22">
+        <v>3.20422080756855</v>
       </c>
     </row>
     <row r="23">
@@ -5718,81 +5492,53 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D23">
+        <v>5.99277326678143</v>
+      </c>
+      <c r="E23">
+        <v>0.517106064131578</v>
+      </c>
+      <c r="F23">
+        <v>-2.16581205540586</v>
+      </c>
+      <c r="G23">
+        <v>-4.77286225333055</v>
       </c>
       <c r="H23">
         <v>1.9929866343406</v>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="I23">
+        <v>-3.05583607385358</v>
+      </c>
+      <c r="J23">
+        <v>-3.05583607385358</v>
       </c>
       <c r="K23">
         <v>3.99857774867471</v>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L23">
+        <v>-6.07727806881682</v>
+      </c>
+      <c r="M23">
+        <v>-0.134902744353604</v>
+      </c>
+      <c r="N23">
+        <v>10.7997826269264</v>
+      </c>
+      <c r="O23">
+        <v>8.24798886137972</v>
+      </c>
+      <c r="P23">
+        <v>-0.24672782331967</v>
+      </c>
+      <c r="Q23">
+        <v>-5.84497141624612</v>
+      </c>
+      <c r="R23">
+        <v>0.112101664963937</v>
+      </c>
+      <c r="S23">
+        <v>-3.34761470772855</v>
       </c>
     </row>
     <row r="24">
@@ -5809,81 +5555,53 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D24">
+        <v>-0.865517957037643</v>
+      </c>
+      <c r="E24">
+        <v>1.53593056697696</v>
+      </c>
+      <c r="F24">
+        <v>1.57074690808372</v>
+      </c>
+      <c r="G24">
+        <v>10.6536072617903</v>
       </c>
       <c r="H24">
         <v>11.5580493725755</v>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="I24">
+        <v>2.40849954847673</v>
+      </c>
+      <c r="J24">
+        <v>2.40849954847673</v>
       </c>
       <c r="K24">
         <v>5.90658890085385</v>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L24">
+        <v>-11.2382387602066</v>
+      </c>
+      <c r="M24">
+        <v>-10.1096906852814</v>
+      </c>
+      <c r="N24">
+        <v>-2.77806564527858</v>
+      </c>
+      <c r="O24">
+        <v>1.13583309548722</v>
+      </c>
+      <c r="P24">
+        <v>2.06529713395707</v>
+      </c>
+      <c r="Q24">
+        <v>-13.034338083299</v>
+      </c>
+      <c r="R24">
+        <v>-11.9286262433148</v>
+      </c>
+      <c r="S24">
+        <v>-4.12689935464596</v>
       </c>
     </row>
     <row r="25">
@@ -5900,81 +5618,53 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D25">
+        <v>3.78110786393069</v>
+      </c>
+      <c r="E25">
+        <v>5.48774575961399</v>
+      </c>
+      <c r="F25">
+        <v>5.58582138597641</v>
+      </c>
+      <c r="G25">
+        <v>3.76666216776007</v>
       </c>
       <c r="H25">
         <v>4.08649128827614</v>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="I25">
+        <v>4.25119332650008</v>
+      </c>
+      <c r="J25">
+        <v>4.25119332650008</v>
       </c>
       <c r="K25">
         <v>2.48232045559289</v>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L25">
+        <v>8.09415475380055</v>
+      </c>
+      <c r="M25">
+        <v>7.58878696984278</v>
+      </c>
+      <c r="N25">
+        <v>2.36160631204012</v>
+      </c>
+      <c r="O25">
+        <v>2.88104477406446</v>
+      </c>
+      <c r="P25">
+        <v>3.88506751575208</v>
+      </c>
+      <c r="Q25">
+        <v>4.0516768566476</v>
+      </c>
+      <c r="R25">
+        <v>3.56520868942891</v>
+      </c>
+      <c r="S25">
+        <v>2.93262807737009</v>
       </c>
     </row>
   </sheetData>
@@ -7460,91 +7150,59 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D21">
+        <v>-9.81002725972002</v>
+      </c>
+      <c r="E21">
+        <v>-13.3819672696904</v>
+      </c>
+      <c r="F21">
+        <v>-8.14977168410478</v>
+      </c>
+      <c r="G21">
+        <v>-13.6380704910772</v>
+      </c>
+      <c r="H21">
+        <v>-3.43012395732717</v>
       </c>
       <c r="I21">
         <v>-11.6707872050536</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J21">
+        <v>3.31059766134347</v>
+      </c>
+      <c r="K21">
+        <v>3.31059766134347</v>
       </c>
       <c r="L21">
         <v>-6.31793996449992</v>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M21">
+        <v>-19.1819779168192</v>
+      </c>
+      <c r="N21">
+        <v>-16.7534073069817</v>
+      </c>
+      <c r="O21">
+        <v>-8.15156287735834</v>
+      </c>
+      <c r="P21">
+        <v>-8.71382147714952</v>
+      </c>
+      <c r="Q21">
+        <v>0.636311694030134</v>
+      </c>
+      <c r="R21">
+        <v>-19.6929808706662</v>
+      </c>
+      <c r="S21">
+        <v>-17.2797658303325</v>
+      </c>
+      <c r="T21">
+        <v>-5.6964426561803</v>
+      </c>
+      <c r="U21">
+        <v>-7.54042695315801</v>
       </c>
     </row>
     <row r="22">
@@ -7561,91 +7219,59 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D22">
+        <v>10.9536314567328</v>
+      </c>
+      <c r="E22">
+        <v>10.7025599885486</v>
+      </c>
+      <c r="F22">
+        <v>9.1273432445663</v>
+      </c>
+      <c r="G22">
+        <v>27.2797543954934</v>
+      </c>
+      <c r="H22">
+        <v>-0.89921055574993</v>
       </c>
       <c r="I22">
         <v>-0.457857875018219</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J22">
+        <v>14.6007709517569</v>
+      </c>
+      <c r="K22">
+        <v>14.6007709517569</v>
       </c>
       <c r="L22">
         <v>1.85057458021192</v>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M22">
+        <v>75.7203450764267</v>
+      </c>
+      <c r="N22">
+        <v>23.1661624074967</v>
+      </c>
+      <c r="O22">
+        <v>11.0635664362215</v>
+      </c>
+      <c r="P22">
+        <v>9.28244036830199</v>
+      </c>
+      <c r="Q22">
+        <v>13.527845904938</v>
+      </c>
+      <c r="R22">
+        <v>54.7817133988125</v>
+      </c>
+      <c r="S22">
+        <v>8.48982593277536</v>
+      </c>
+      <c r="T22">
+        <v>1.44346659338355</v>
+      </c>
+      <c r="U22">
+        <v>8.69114921032221</v>
       </c>
     </row>
     <row r="23">
@@ -7662,91 +7288,59 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D23">
+        <v>13.07993120299</v>
+      </c>
+      <c r="E23">
+        <v>11.3599363030651</v>
+      </c>
+      <c r="F23">
+        <v>0.517106064131578</v>
+      </c>
+      <c r="G23">
+        <v>-0.684165561946082</v>
+      </c>
+      <c r="H23">
+        <v>-6.58758208241558</v>
       </c>
       <c r="I23">
         <v>4.36701656673211</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J23">
+        <v>-1.79615121357592</v>
+      </c>
+      <c r="K23">
+        <v>-1.79615121357592</v>
       </c>
       <c r="L23">
         <v>3.63060276374092</v>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M23">
+        <v>-3.45173135601112</v>
+      </c>
+      <c r="N23">
+        <v>19.6203416468141</v>
+      </c>
+      <c r="O23">
+        <v>13.8306058448039</v>
+      </c>
+      <c r="P23">
+        <v>12.4980022817821</v>
+      </c>
+      <c r="Q23">
+        <v>0.979727476773307</v>
+      </c>
+      <c r="R23">
+        <v>-4.38846384667034</v>
+      </c>
+      <c r="S23">
+        <v>18.459758840534</v>
+      </c>
+      <c r="T23">
+        <v>10.7870497505327</v>
+      </c>
+      <c r="U23">
+        <v>7.45854345452925</v>
       </c>
     </row>
     <row r="24">
@@ -7763,91 +7357,59 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D24">
+        <v>-12.3264328654353</v>
+      </c>
+      <c r="E24">
+        <v>-13.0913586031985</v>
+      </c>
+      <c r="F24">
+        <v>1.53593056697696</v>
+      </c>
+      <c r="G24">
+        <v>-15.3567202124469</v>
+      </c>
+      <c r="H24">
+        <v>10.2185477821095</v>
       </c>
       <c r="I24">
         <v>4.11449131743504</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J24">
+        <v>-1.48173362664032</v>
+      </c>
+      <c r="K24">
+        <v>-1.48173362664032</v>
       </c>
       <c r="L24">
         <v>0.0384891748981708</v>
       </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M24">
+        <v>-36.8380108521467</v>
+      </c>
+      <c r="N24">
+        <v>-27.1033000274007</v>
+      </c>
+      <c r="O24">
+        <v>-11.9998346654394</v>
+      </c>
+      <c r="P24">
+        <v>-9.89472032385233</v>
+      </c>
+      <c r="Q24">
+        <v>-3.30186552075882</v>
+      </c>
+      <c r="R24">
+        <v>-34.681274372038</v>
+      </c>
+      <c r="S24">
+        <v>-24.6141610019907</v>
+      </c>
+      <c r="T24">
+        <v>-14.4060226645845</v>
+      </c>
+      <c r="U24">
+        <v>-13.1247961523505</v>
       </c>
     </row>
     <row r="25">
@@ -7864,91 +7426,59 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D25">
+        <v>1.72867593550896</v>
+      </c>
+      <c r="E25">
+        <v>5.51158842847319</v>
+      </c>
+      <c r="F25">
+        <v>5.48774575961399</v>
+      </c>
+      <c r="G25">
+        <v>5.73325625254468</v>
+      </c>
+      <c r="H25">
+        <v>6.99084137342969</v>
       </c>
       <c r="I25">
         <v>2.31934672136751</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J25">
+        <v>4.20971444765637</v>
+      </c>
+      <c r="K25">
+        <v>4.20971444765637</v>
       </c>
       <c r="L25">
         <v>1.52173879485957</v>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M25">
+        <v>10.0715745156174</v>
+      </c>
+      <c r="N25">
+        <v>8.02181188680047</v>
+      </c>
+      <c r="O25">
+        <v>0.133530517309444</v>
+      </c>
+      <c r="P25">
+        <v>0.463472917094809</v>
+      </c>
+      <c r="Q25">
+        <v>3.45448211394401</v>
+      </c>
+      <c r="R25">
+        <v>6.39613892647528</v>
+      </c>
+      <c r="S25">
+        <v>4.41482058537204</v>
+      </c>
+      <c r="T25">
+        <v>0.0226023114699325</v>
+      </c>
+      <c r="U25">
+        <v>3.93004461997615</v>
       </c>
     </row>
   </sheetData>
@@ -9288,25 +8818,17 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D21">
+        <v>1.58691769995684</v>
+      </c>
+      <c r="E21">
+        <v>1.79308748609151</v>
+      </c>
+      <c r="F21">
+        <v>1.82321819540689</v>
+      </c>
+      <c r="G21">
+        <v>1.36389309432053</v>
       </c>
       <c r="H21">
         <v>2.49633216113152</v>
@@ -9316,53 +8838,35 @@
           <t/>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J21">
+        <v>1.42004212868474</v>
       </c>
       <c r="K21">
         <v>1.4566295307954</v>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L21">
+        <v>1.36618854378898</v>
+      </c>
+      <c r="M21">
+        <v>1.37751594738923</v>
+      </c>
+      <c r="N21">
+        <v>1.44304026444907</v>
+      </c>
+      <c r="O21">
+        <v>1.66050393749557</v>
+      </c>
+      <c r="P21">
+        <v>1.47171261606599</v>
+      </c>
+      <c r="Q21">
+        <v>0.928298452343848</v>
+      </c>
+      <c r="R21">
+        <v>0.935995202019429</v>
+      </c>
+      <c r="S21">
+        <v>1.2309838899891</v>
       </c>
     </row>
     <row r="22">
@@ -9379,25 +8883,17 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D22">
+        <v>1.72041144441653</v>
+      </c>
+      <c r="E22">
+        <v>1.95674873562245</v>
+      </c>
+      <c r="F22">
+        <v>2.08773517870931</v>
+      </c>
+      <c r="G22">
+        <v>1.25044040940981</v>
       </c>
       <c r="H22">
         <v>2.43900799041786</v>
@@ -9407,53 +8903,35 @@
           <t/>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J22">
+        <v>1.43834980450519</v>
       </c>
       <c r="K22">
         <v>1.54022877691862</v>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L22">
+        <v>2.00540222167942</v>
+      </c>
+      <c r="M22">
+        <v>1.76294128139568</v>
+      </c>
+      <c r="N22">
+        <v>1.55548134475901</v>
+      </c>
+      <c r="O22">
+        <v>1.73789511838111</v>
+      </c>
+      <c r="P22">
+        <v>1.50271616869949</v>
+      </c>
+      <c r="Q22">
+        <v>1.33451829656892</v>
+      </c>
+      <c r="R22">
+        <v>1.17316983613838</v>
+      </c>
+      <c r="S22">
+        <v>1.27042733192995</v>
       </c>
     </row>
     <row r="23">
@@ -9470,25 +8948,17 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D23">
+        <v>1.82351180153617</v>
+      </c>
+      <c r="E23">
+        <v>1.96686720199417</v>
+      </c>
+      <c r="F23">
+        <v>2.04251875852387</v>
+      </c>
+      <c r="G23">
+        <v>1.1907586111087</v>
       </c>
       <c r="H23">
         <v>2.48761709367739</v>
@@ -9498,53 +8968,35 @@
           <t/>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J23">
+        <v>1.39439619231092</v>
       </c>
       <c r="K23">
         <v>1.60181602207118</v>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L23">
+        <v>1.88352835226973</v>
+      </c>
+      <c r="M23">
+        <v>1.76056302522573</v>
+      </c>
+      <c r="N23">
+        <v>1.72346994879537</v>
+      </c>
+      <c r="O23">
+        <v>1.88123651416765</v>
+      </c>
+      <c r="P23">
+        <v>1.49900854980578</v>
+      </c>
+      <c r="Q23">
+        <v>1.25651608358989</v>
+      </c>
+      <c r="R23">
+        <v>1.17448497905755</v>
+      </c>
+      <c r="S23">
+        <v>1.22789831971526</v>
       </c>
     </row>
     <row r="24">
@@ -9561,25 +9013,17 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D24">
+        <v>1.80772897944517</v>
+      </c>
+      <c r="E24">
+        <v>1.99707691656145</v>
+      </c>
+      <c r="F24">
+        <v>2.07460155877042</v>
+      </c>
+      <c r="G24">
+        <v>1.31761735697217</v>
       </c>
       <c r="H24">
         <v>2.77513710556525</v>
@@ -9589,53 +9033,35 @@
           <t/>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J24">
+        <v>1.4279802183067</v>
       </c>
       <c r="K24">
         <v>1.69642870944293</v>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L24">
+        <v>1.67185293892547</v>
+      </c>
+      <c r="M24">
+        <v>1.58257554905598</v>
+      </c>
+      <c r="N24">
+        <v>1.67559082224118</v>
+      </c>
+      <c r="O24">
+        <v>1.90260422109995</v>
+      </c>
+      <c r="P24">
+        <v>1.52996753042269</v>
+      </c>
+      <c r="Q24">
+        <v>1.09273752918376</v>
+      </c>
+      <c r="R24">
+        <v>1.0343850556219</v>
+      </c>
+      <c r="S24">
+        <v>1.17722419188322</v>
       </c>
     </row>
     <row r="25">
@@ -9652,25 +9078,17 @@
           <t>economia_total</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D25">
+        <v>1.87608116204553</v>
+      </c>
+      <c r="E25">
+        <v>2.10667142036628</v>
+      </c>
+      <c r="F25">
+        <v>2.19048509631401</v>
+      </c>
+      <c r="G25">
+        <v>1.36724755147308</v>
       </c>
       <c r="H25">
         <v>2.88854284162189</v>
@@ -9680,53 +9098,35 @@
           <t/>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="J25">
+        <v>1.4886864180511</v>
       </c>
       <c r="K25">
         <v>1.73853950631198</v>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L25">
+        <v>1.80717530305806</v>
+      </c>
+      <c r="M25">
+        <v>1.70267383611066</v>
+      </c>
+      <c r="N25">
+        <v>1.7151616808632</v>
+      </c>
+      <c r="O25">
+        <v>1.95741910058308</v>
+      </c>
+      <c r="P25">
+        <v>1.5894078019487</v>
+      </c>
+      <c r="Q25">
+        <v>1.1370117227576</v>
+      </c>
+      <c r="R25">
+        <v>1.07126304150709</v>
+      </c>
+      <c r="S25">
+        <v>1.21174779906798</v>
       </c>
     </row>
   </sheetData>
@@ -11190,30 +10590,20 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D21">
+        <v>1.05794863216347</v>
+      </c>
+      <c r="E21">
+        <v>1.1030793747383</v>
+      </c>
+      <c r="F21">
+        <v>1.79308748609151</v>
+      </c>
+      <c r="G21">
+        <v>1.1030391881238</v>
+      </c>
+      <c r="H21">
+        <v>1.27093528739059</v>
       </c>
       <c r="I21">
         <v>1.70181507627533</v>
@@ -11223,58 +10613,38 @@
           <t/>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="K21">
+        <v>1.84015021003721</v>
       </c>
       <c r="L21">
         <v>0.827664818684173</v>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M21">
+        <v>0.719109192999619</v>
+      </c>
+      <c r="N21">
+        <v>0.823352679730219</v>
+      </c>
+      <c r="O21">
+        <v>1.03932958118967</v>
+      </c>
+      <c r="P21">
+        <v>1.10588158273995</v>
+      </c>
+      <c r="Q21">
+        <v>1.62277998967081</v>
+      </c>
+      <c r="R21">
+        <v>0.44313412636145</v>
+      </c>
+      <c r="S21">
+        <v>0.507371723197819</v>
+      </c>
+      <c r="T21">
+        <v>0.615184358429016</v>
+      </c>
+      <c r="U21">
+        <v>1.33276097985171</v>
       </c>
     </row>
     <row r="22">
@@ -11291,30 +10661,20 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D22">
+        <v>1.1738324263322</v>
+      </c>
+      <c r="E22">
+        <v>1.22113710654098</v>
+      </c>
+      <c r="F22">
+        <v>1.95674873562245</v>
+      </c>
+      <c r="G22">
+        <v>1.40394556953002</v>
+      </c>
+      <c r="H22">
+        <v>1.25950690312962</v>
       </c>
       <c r="I22">
         <v>1.69402318193035</v>
@@ -11324,58 +10684,38 @@
           <t/>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="K22">
+        <v>2.10882632737302</v>
       </c>
       <c r="L22">
         <v>0.842981373428099</v>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M22">
+        <v>1.26362115541524</v>
+      </c>
+      <c r="N22">
+        <v>1.014091898703</v>
+      </c>
+      <c r="O22">
+        <v>1.15431649989589</v>
+      </c>
+      <c r="P22">
+        <v>1.20853438120182</v>
+      </c>
+      <c r="Q22">
+        <v>1.84230716604965</v>
+      </c>
+      <c r="R22">
+        <v>0.685890593437112</v>
+      </c>
+      <c r="S22">
+        <v>0.550446699329437</v>
+      </c>
+      <c r="T22">
+        <v>0.62406433913066</v>
+      </c>
+      <c r="U22">
+        <v>1.44859322522757</v>
       </c>
     </row>
     <row r="23">
@@ -11392,30 +10732,20 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D23">
+        <v>1.32736890013484</v>
+      </c>
+      <c r="E23">
+        <v>1.35985750401713</v>
+      </c>
+      <c r="F23">
+        <v>1.96686720199417</v>
+      </c>
+      <c r="G23">
+        <v>1.39434025743483</v>
+      </c>
+      <c r="H23">
+        <v>1.17653585205227</v>
       </c>
       <c r="I23">
         <v>1.76800145492953</v>
@@ -11425,58 +10755,38 @@
           <t/>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="K23">
+        <v>2.0709486177017</v>
       </c>
       <c r="L23">
         <v>0.873586678469601</v>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M23">
+        <v>1.22000434777258</v>
+      </c>
+      <c r="N23">
+        <v>1.21306019384119</v>
+      </c>
+      <c r="O23">
+        <v>1.31396546519803</v>
+      </c>
+      <c r="P23">
+        <v>1.35957703574055</v>
+      </c>
+      <c r="Q23">
+        <v>1.860356755562</v>
+      </c>
+      <c r="R23">
+        <v>0.655790532716411</v>
+      </c>
+      <c r="S23">
+        <v>0.65205783257133</v>
+      </c>
+      <c r="T23">
+        <v>0.691382469868017</v>
+      </c>
+      <c r="U23">
+        <v>1.55663718041054</v>
       </c>
     </row>
     <row r="24">
@@ -11493,30 +10803,20 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D24">
+        <v>1.16375166378305</v>
+      </c>
+      <c r="E24">
+        <v>1.18183368167374</v>
+      </c>
+      <c r="F24">
+        <v>1.99707691656145</v>
+      </c>
+      <c r="G24">
+        <v>1.18021532529105</v>
+      </c>
+      <c r="H24">
+        <v>1.29676073026788</v>
       </c>
       <c r="I24">
         <v>1.84074572128473</v>
@@ -11526,58 +10826,38 @@
           <t/>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="K24">
+        <v>2.04026267564277</v>
       </c>
       <c r="L24">
         <v>0.873922914774164</v>
       </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M24">
+        <v>0.770579013743455</v>
+      </c>
+      <c r="N24">
+        <v>0.884280849991444</v>
+      </c>
+      <c r="O24">
+        <v>1.1562917818133</v>
+      </c>
+      <c r="P24">
+        <v>1.2250506904667</v>
+      </c>
+      <c r="Q24">
+        <v>1.79893027728699</v>
+      </c>
+      <c r="R24">
+        <v>0.428354018759183</v>
+      </c>
+      <c r="S24">
+        <v>0.491559267836132</v>
+      </c>
+      <c r="T24">
+        <v>0.591781754559866</v>
+      </c>
+      <c r="U24">
+        <v>1.35233172364996</v>
       </c>
     </row>
     <row r="25">
@@ -11594,30 +10874,20 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D25">
+        <v>1.18386915874396</v>
+      </c>
+      <c r="E25">
+        <v>1.24697149011667</v>
+      </c>
+      <c r="F25">
+        <v>2.10667142036628</v>
+      </c>
+      <c r="G25">
+        <v>1.24788009422179</v>
+      </c>
+      <c r="H25">
+        <v>1.38741521591383</v>
       </c>
       <c r="I25">
         <v>1.88343899682007</v>
@@ -11627,58 +10897,38 @@
           <t/>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="K25">
+        <v>2.12615190826944</v>
       </c>
       <c r="L25">
         <v>0.88722173880545</v>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="M25">
+        <v>0.848188453314337</v>
+      </c>
+      <c r="N25">
+        <v>0.955216196328758</v>
+      </c>
+      <c r="O25">
+        <v>1.15783578421116</v>
+      </c>
+      <c r="P25">
+        <v>1.2307284686377</v>
+      </c>
+      <c r="Q25">
+        <v>1.86107400195819</v>
+      </c>
+      <c r="R25">
+        <v>0.455752136896161</v>
+      </c>
+      <c r="S25">
+        <v>0.513260727581866</v>
+      </c>
+      <c r="T25">
+        <v>0.591915510915254</v>
+      </c>
+      <c r="U25">
+        <v>1.40547896379949</v>
       </c>
     </row>
   </sheetData>
@@ -43839,89 +43089,59 @@
       <c r="D21">
         <v>4.2</v>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E21">
+        <v>3.07205708091106</v>
       </c>
       <c r="F21">
         <v>3.14718882182406</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G21">
+        <v>587584826815.644</v>
+      </c>
+      <c r="H21">
+        <v>272887536854.195</v>
+      </c>
+      <c r="I21">
+        <v>255648452296.867</v>
+      </c>
+      <c r="J21">
+        <v>23590077148.2075</v>
       </c>
       <c r="K21">
         <v>141640226606.943</v>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L21">
+        <v>339498352861.141</v>
+      </c>
+      <c r="M21">
+        <v>339498352861.141</v>
       </c>
       <c r="N21">
         <v>570247.155233905</v>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="O21">
+        <v>90418148541.7169</v>
+      </c>
+      <c r="P21">
+        <v>107657233099.045</v>
+      </c>
+      <c r="Q21">
+        <v>314697289961.45</v>
+      </c>
+      <c r="R21">
+        <v>108651789659.141</v>
+      </c>
+      <c r="S21">
+        <v>448150142520.282</v>
+      </c>
+      <c r="T21">
+        <v>0.201758607133824</v>
+      </c>
+      <c r="U21">
+        <v>0.240225814709347</v>
+      </c>
+      <c r="V21">
+        <v>478542.565884894</v>
       </c>
     </row>
     <row r="22">
@@ -43941,89 +43161,59 @@
       <c r="D22">
         <v>4.2</v>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E22">
+        <v>3.41225692935307</v>
       </c>
       <c r="F22">
         <v>3.39769972910033</v>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G22">
+        <v>637013287233.881</v>
+      </c>
+      <c r="H22">
+        <v>297794919014.519</v>
+      </c>
+      <c r="I22">
+        <v>292738558987.256</v>
+      </c>
+      <c r="J22">
+        <v>21627784354.982</v>
       </c>
       <c r="K22">
         <v>138387691284.777</v>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L22">
+        <v>343875283418.486</v>
+      </c>
+      <c r="M22">
+        <v>343875283418.486</v>
       </c>
       <c r="N22">
         <v>602974.92250321</v>
       </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="O22">
+        <v>132723083347.496</v>
+      </c>
+      <c r="P22">
+        <v>137779443374.76</v>
+      </c>
+      <c r="Q22">
+        <v>339218368219.362</v>
+      </c>
+      <c r="R22">
+        <v>113715728453.367</v>
+      </c>
+      <c r="S22">
+        <v>457591011871.852</v>
+      </c>
+      <c r="T22">
+        <v>0.290047400198204</v>
+      </c>
+      <c r="U22">
+        <v>0.301097355062002</v>
+      </c>
+      <c r="V22">
+        <v>493876.126354051</v>
       </c>
     </row>
     <row r="23">
@@ -44043,89 +43233,59 @@
       <c r="D23">
         <v>4.2</v>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E23">
+        <v>3.61661765851799</v>
       </c>
       <c r="F23">
         <v>3.70010931039399</v>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G23">
+        <v>675188049217.079</v>
+      </c>
+      <c r="H23">
+        <v>299334834599.419</v>
+      </c>
+      <c r="I23">
+        <v>286398391985.888</v>
+      </c>
+      <c r="J23">
+        <v>20595519999.2713</v>
       </c>
       <c r="K23">
         <v>141145739475.656</v>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L23">
+        <v>333367018458.718</v>
+      </c>
+      <c r="M23">
+        <v>333367018458.718</v>
       </c>
       <c r="N23">
         <v>627085.343584512</v>
       </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="O23">
+        <v>124657132510.961</v>
+      </c>
+      <c r="P23">
+        <v>137593575124.492</v>
+      </c>
+      <c r="Q23">
+        <v>375853214617.66</v>
+      </c>
+      <c r="R23">
+        <v>123094989069.837</v>
+      </c>
+      <c r="S23">
+        <v>456462007528.555</v>
+      </c>
+      <c r="T23">
+        <v>0.273094212563054</v>
+      </c>
+      <c r="U23">
+        <v>0.301434890210189</v>
+      </c>
+      <c r="V23">
+        <v>477343.056510262</v>
       </c>
     </row>
     <row r="24">
@@ -44145,89 +43305,59 @@
       <c r="D24">
         <v>4.2</v>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E24">
+        <v>3.76320113204531</v>
       </c>
       <c r="F24">
         <v>3.88878855567701</v>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G24">
+        <v>669344175407.333</v>
+      </c>
+      <c r="H24">
+        <v>303932409821.641</v>
+      </c>
+      <c r="I24">
+        <v>290896985872.808</v>
+      </c>
+      <c r="J24">
+        <v>22789685813.5172</v>
       </c>
       <c r="K24">
         <v>157459433731.539</v>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L24">
+        <v>341396161593.066</v>
+      </c>
+      <c r="M24">
+        <v>341396161593.066</v>
       </c>
       <c r="N24">
         <v>664124.696887556</v>
       </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="O24">
+        <v>110647866327.752</v>
+      </c>
+      <c r="P24">
+        <v>123683290276.586</v>
+      </c>
+      <c r="Q24">
+        <v>365411765585.691</v>
+      </c>
+      <c r="R24">
+        <v>124493142694.579</v>
+      </c>
+      <c r="S24">
+        <v>465889304287.645</v>
+      </c>
+      <c r="T24">
+        <v>0.237498189611662</v>
+      </c>
+      <c r="U24">
+        <v>0.265477848790069</v>
+      </c>
+      <c r="V24">
+        <v>457643.588991693</v>
       </c>
     </row>
     <row r="25">
@@ -44247,89 +43377,59 @@
       <c r="D25">
         <v>4.2</v>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E25">
+        <v>3.92076753234211</v>
       </c>
       <c r="F25">
         <v>4.1023240340288</v>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="G25">
+        <v>694652800660.422</v>
+      </c>
+      <c r="H25">
+        <v>320611447753.721</v>
+      </c>
+      <c r="I25">
+        <v>307145971920.852</v>
+      </c>
+      <c r="J25">
+        <v>23648096287.2063</v>
       </c>
       <c r="K25">
         <v>163893999773.547</v>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="L25">
+        <v>355909572431.638</v>
+      </c>
+      <c r="M25">
+        <v>355909572431.638</v>
       </c>
       <c r="N25">
         <v>680610.40008904</v>
       </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="O25">
+        <v>119603875860.099</v>
+      </c>
+      <c r="P25">
+        <v>133069351692.968</v>
+      </c>
+      <c r="Q25">
+        <v>374041352906.7</v>
+      </c>
+      <c r="R25">
+        <v>128079845876.249</v>
+      </c>
+      <c r="S25">
+        <v>483989418307.887</v>
+      </c>
+      <c r="T25">
+        <v>0.247120848795115</v>
+      </c>
+      <c r="U25">
+        <v>0.274942688123641</v>
+      </c>
+      <c r="V25">
+        <v>471064.573376748</v>
       </c>
     </row>
   </sheetData>

</xml_diff>